<commit_message>
배포판 자동 동기화 — 10b8ae2 (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/sample_input.xlsx
+++ b/sample_input.xlsx
@@ -751,7 +751,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
     </row>

</xml_diff>